<commit_message>
Melhorias no sistema, tabelas e visuais aprimorados
</commit_message>
<xml_diff>
--- a/output/Planilha_Final.xlsx
+++ b/output/Planilha_Final.xlsx
@@ -1322,7 +1322,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>FDSA</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
@@ -5011,17 +5011,17 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 6M</t>
         </is>
       </c>
       <c r="C7" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D7" s="70" t="n">
-        <v>3236.79</v>
+        <v>352.84</v>
       </c>
       <c r="E7" s="70" t="n">
-        <v>647.36</v>
+        <v>176.42</v>
       </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="72" t="inlineStr">
@@ -5041,17 +5041,17 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="69" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 6M</t>
+          <t>XLEGENDA SISTEMATIZAÇÃO</t>
         </is>
       </c>
       <c r="C8" s="70" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D8" s="70" t="n">
-        <v>352.84</v>
+        <v>168.81</v>
       </c>
       <c r="E8" s="70" t="n">
-        <v>176.42</v>
+        <v>16.88</v>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
@@ -5067,17 +5067,17 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="69" t="inlineStr">
         <is>
-          <t>TALHÕES</t>
+          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
         </is>
       </c>
       <c r="C9" s="70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="70" t="n">
-        <v>3031</v>
+        <v>18.96</v>
       </c>
       <c r="E9" s="70" t="n">
-        <v>1010.33</v>
+        <v>18.96</v>
       </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
@@ -5089,17 +5089,17 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
-          <t>NUMERAÇÕES DOS TALHÕES</t>
+          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
         </is>
       </c>
       <c r="C10" s="70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="70" t="n">
-        <v>81.34</v>
+        <v>143.06</v>
       </c>
       <c r="E10" s="70" t="n">
-        <v>81.34</v>
+        <v>71.53</v>
       </c>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
@@ -5111,17 +5111,17 @@
       <c r="A11" s="5" t="n"/>
       <c r="B11" s="69" t="inlineStr">
         <is>
-          <t>XLEGENDA SISTEMATIZAÇÃO</t>
+          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
         </is>
       </c>
       <c r="C11" s="70" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D11" s="70" t="n">
-        <v>168.81</v>
+        <v>2585.6</v>
       </c>
       <c r="E11" s="70" t="n">
-        <v>16.88</v>
+        <v>2585.6</v>
       </c>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
@@ -5131,20 +5131,6 @@
     </row>
     <row r="12" ht="18.75" customHeight="1" s="39">
       <c r="A12" s="5" t="n"/>
-      <c r="B12" s="69" t="inlineStr">
-        <is>
-          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
-        </is>
-      </c>
-      <c r="C12" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="70" t="n">
-        <v>18.96</v>
-      </c>
-      <c r="E12" s="70" t="n">
-        <v>18.96</v>
-      </c>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
@@ -5153,38 +5139,14 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" s="39">
       <c r="A13" s="5" t="n"/>
-      <c r="B13" s="69" t="inlineStr">
-        <is>
-          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
-        </is>
-      </c>
-      <c r="C13" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="70" t="n">
-        <v>143.06</v>
-      </c>
-      <c r="E13" s="70" t="n">
-        <v>71.53</v>
-      </c>
       <c r="J13" s="11" t="n"/>
     </row>
     <row r="14" ht="18.75" customHeight="1" s="39">
       <c r="A14" s="5" t="n"/>
-      <c r="B14" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="70" t="n">
-        <v>2585.6</v>
-      </c>
-      <c r="E14" s="70" t="n">
-        <v>2585.6</v>
-      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
       <c r="J14" s="11" t="n"/>
     </row>
     <row r="15" ht="18.75" customHeight="1" s="39">
@@ -5340,7 +5302,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>FDSA</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Atualização na imterface e correções
</commit_message>
<xml_diff>
--- a/output/Planilha_Final.xlsx
+++ b/output/Planilha_Final.xlsx
@@ -1322,7 +1322,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>DAS</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
@@ -5011,17 +5011,17 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="69" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 6M</t>
+          <t>XLEGENDA SISTEMATIZAÇÃO</t>
         </is>
       </c>
       <c r="C7" s="70" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D7" s="70" t="n">
-        <v>352.84</v>
+        <v>168.81</v>
       </c>
       <c r="E7" s="70" t="n">
-        <v>176.42</v>
+        <v>16.88</v>
       </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="72" t="inlineStr">
@@ -5041,17 +5041,17 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="69" t="inlineStr">
         <is>
-          <t>XLEGENDA SISTEMATIZAÇÃO</t>
+          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
         </is>
       </c>
       <c r="C8" s="70" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D8" s="70" t="n">
-        <v>168.81</v>
+        <v>18.96</v>
       </c>
       <c r="E8" s="70" t="n">
-        <v>16.88</v>
+        <v>18.96</v>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
@@ -5067,17 +5067,17 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="69" t="inlineStr">
         <is>
-          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
+          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
         </is>
       </c>
       <c r="C9" s="70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" s="70" t="n">
-        <v>18.96</v>
+        <v>143.06</v>
       </c>
       <c r="E9" s="70" t="n">
-        <v>18.96</v>
+        <v>71.53</v>
       </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
@@ -5089,17 +5089,17 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
-          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
+          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
         </is>
       </c>
       <c r="C10" s="70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="70" t="n">
-        <v>143.06</v>
+        <v>2585.6</v>
       </c>
       <c r="E10" s="70" t="n">
-        <v>71.53</v>
+        <v>2585.6</v>
       </c>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
@@ -5109,20 +5109,6 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" s="39">
       <c r="A11" s="5" t="n"/>
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="70" t="n">
-        <v>2585.6</v>
-      </c>
-      <c r="E11" s="70" t="n">
-        <v>2585.6</v>
-      </c>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
@@ -5302,7 +5288,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>DSA</t>
+          <t>DAS</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Correção de escala e janelas
</commit_message>
<xml_diff>
--- a/output/Planilha_Final.xlsx
+++ b/output/Planilha_Final.xlsx
@@ -1322,7 +1322,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>DAS</t>
+          <t>DSADSA</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
@@ -5011,17 +5011,17 @@
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="69" t="inlineStr">
         <is>
-          <t>XLEGENDA SISTEMATIZAÇÃO</t>
+          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 6M</t>
         </is>
       </c>
       <c r="C7" s="70" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D7" s="70" t="n">
-        <v>168.81</v>
+        <v>352.84</v>
       </c>
       <c r="E7" s="70" t="n">
-        <v>16.88</v>
+        <v>176.42</v>
       </c>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="72" t="inlineStr">
@@ -5041,17 +5041,17 @@
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="69" t="inlineStr">
         <is>
-          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
+          <t>XLEGENDA SISTEMATIZAÇÃO</t>
         </is>
       </c>
       <c r="C8" s="70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D8" s="70" t="n">
-        <v>18.96</v>
+        <v>168.81</v>
       </c>
       <c r="E8" s="70" t="n">
-        <v>18.96</v>
+        <v>16.88</v>
       </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
@@ -5067,17 +5067,17 @@
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="69" t="inlineStr">
         <is>
-          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
+          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
         </is>
       </c>
       <c r="C9" s="70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="70" t="n">
-        <v>143.06</v>
+        <v>18.96</v>
       </c>
       <c r="E9" s="70" t="n">
-        <v>71.53</v>
+        <v>18.96</v>
       </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
@@ -5089,17 +5089,17 @@
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
+          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
         </is>
       </c>
       <c r="C10" s="70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="70" t="n">
-        <v>2585.6</v>
+        <v>143.06</v>
       </c>
       <c r="E10" s="70" t="n">
-        <v>2585.6</v>
+        <v>71.53</v>
       </c>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
@@ -5109,6 +5109,20 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" s="39">
       <c r="A11" s="5" t="n"/>
+      <c r="B11" s="69" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="70" t="n">
+        <v>2585.6</v>
+      </c>
+      <c r="E11" s="70" t="n">
+        <v>2585.6</v>
+      </c>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
@@ -5288,7 +5302,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>DAS</t>
+          <t>DSADSA</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Imagens para o README
</commit_message>
<xml_diff>
--- a/output/Planilha_Final.xlsx
+++ b/output/Planilha_Final.xlsx
@@ -274,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -416,12 +416,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1322,7 +1316,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>DSADSA</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
@@ -4919,144 +4913,74 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" s="39">
       <c r="A4" s="5" t="n"/>
-      <c r="B4" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CURVA EMBUTIDA</t>
-        </is>
-      </c>
-      <c r="C4" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" s="70" t="n">
-        <v>1545.45</v>
-      </c>
-      <c r="E4" s="70" t="n">
-        <v>309.09</v>
-      </c>
       <c r="F4" s="6" t="n"/>
-      <c r="G4" s="71" t="inlineStr">
+      <c r="G4" s="69" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="H4" s="71" t="n">
+      <c r="H4" s="69" t="n">
         <v>0.24</v>
       </c>
-      <c r="I4" s="71" t="n">
+      <c r="I4" s="69" t="n">
         <v>0.1</v>
       </c>
       <c r="J4" s="11" t="n"/>
     </row>
     <row r="5" ht="18.75" customHeight="1" s="39">
       <c r="A5" s="5" t="n"/>
-      <c r="B5" s="69" t="inlineStr">
-        <is>
-          <t>REDE</t>
-        </is>
-      </c>
-      <c r="C5" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="70" t="n">
-        <v>118.93</v>
-      </c>
-      <c r="E5" s="70" t="n">
-        <v>118.93</v>
-      </c>
       <c r="F5" s="6" t="n"/>
-      <c r="G5" s="71" t="inlineStr">
+      <c r="G5" s="69" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="H5" s="71" t="n">
+      <c r="H5" s="69" t="n">
         <v>17.2</v>
       </c>
-      <c r="I5" s="71" t="n">
+      <c r="I5" s="69" t="n">
         <v>7.11</v>
       </c>
       <c r="J5" s="11" t="n"/>
     </row>
     <row r="6" ht="18.75" customHeight="1" s="39">
       <c r="A6" s="5" t="n"/>
-      <c r="B6" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 7.5M</t>
-        </is>
-      </c>
-      <c r="C6" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="70" t="n">
-        <v>237.86</v>
-      </c>
-      <c r="E6" s="70" t="n">
-        <v>118.93</v>
-      </c>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="71" t="inlineStr">
+      <c r="G6" s="69" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="H6" s="71" t="n">
+      <c r="H6" s="69" t="n">
         <v>4.24</v>
       </c>
-      <c r="I6" s="71" t="n">
+      <c r="I6" s="69" t="n">
         <v>1.75</v>
       </c>
       <c r="J6" s="35" t="n"/>
     </row>
     <row r="7" ht="18.75" customHeight="1" s="39">
       <c r="A7" s="5" t="n"/>
-      <c r="B7" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 6M</t>
-        </is>
-      </c>
-      <c r="C7" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="70" t="n">
-        <v>352.84</v>
-      </c>
-      <c r="E7" s="70" t="n">
-        <v>176.42</v>
-      </c>
       <c r="F7" s="6" t="n"/>
-      <c r="G7" s="72" t="inlineStr">
+      <c r="G7" s="70" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="H7" s="73" t="n">
+      <c r="H7" s="71" t="n">
         <v>21.69</v>
       </c>
-      <c r="I7" s="73" t="n">
+      <c r="I7" s="71" t="n">
         <v>8.960000000000001</v>
       </c>
       <c r="J7" s="11" t="n"/>
     </row>
     <row r="8" ht="18.75" customHeight="1" s="39">
       <c r="A8" s="5" t="n"/>
-      <c r="B8" s="69" t="inlineStr">
-        <is>
-          <t>XLEGENDA SISTEMATIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" s="70" t="n">
-        <v>168.81</v>
-      </c>
-      <c r="E8" s="70" t="n">
-        <v>16.88</v>
-      </c>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-      <c r="I8" s="74" t="inlineStr">
+      <c r="I8" s="72" t="inlineStr">
         <is>
           <t>*Alqueires Paulistas</t>
         </is>
@@ -5065,20 +4989,6 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" s="39">
       <c r="A9" s="5" t="n"/>
-      <c r="B9" s="69" t="inlineStr">
-        <is>
-          <t>TRANSFORMAÇÃO DE EMBUTIDA P- BASE LARGA</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="70" t="n">
-        <v>18.96</v>
-      </c>
-      <c r="E9" s="70" t="n">
-        <v>18.96</v>
-      </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
@@ -5087,20 +4997,6 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" s="39">
       <c r="A10" s="5" t="n"/>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>CONSTRUÇÃO DE TERRAÇO BASE LARGA</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="70" t="n">
-        <v>143.06</v>
-      </c>
-      <c r="E10" s="70" t="n">
-        <v>71.53</v>
-      </c>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
@@ -5109,20 +5005,6 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" s="39">
       <c r="A11" s="5" t="n"/>
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO-LIMPEZA DE CARREADOR 5M</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="70" t="n">
-        <v>2585.6</v>
-      </c>
-      <c r="E11" s="70" t="n">
-        <v>2585.6</v>
-      </c>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
@@ -5302,7 +5184,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>DSADSA</t>
+          <t>DSA</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">
@@ -5390,7 +5272,7 @@
       <c r="H31" s="23" t="n">
         <v>0.1</v>
       </c>
-      <c r="I31" s="75" t="n"/>
+      <c r="I31" s="73" t="n"/>
       <c r="J31" s="60" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="39">

</xml_diff>